<commit_message>
animation + tuteur + changment de mdp
</commit_message>
<xml_diff>
--- a/docs/modele-import/modele-import-ifspa.xlsx
+++ b/docs/modele-import/modele-import-ifspa.xlsx
@@ -111,6 +111,15 @@
     <t>Adresse</t>
   </si>
   <si>
+    <t>Tuteur</t>
+  </si>
+  <si>
+    <t>Téléphone tuteur</t>
+  </si>
+  <si>
+    <t>Profession tuteur</t>
+  </si>
+  <si>
     <t>Filière *</t>
   </si>
   <si>
@@ -144,6 +153,12 @@
     <t>En texte, ex. 034 12 345 67.</t>
   </si>
   <si>
+    <t>Nom du tuteur, facultatif. Obligatoire si son téléphone ou sa profession est rempli.</t>
+  </si>
+  <si>
+    <t>En texte, ex. 033 12 345 67.</t>
+  </si>
+  <si>
     <t>Code de la filière : IF ou SF.</t>
   </si>
   <si>
@@ -183,6 +198,15 @@
     <t>Lot II A 12 Tanambao V</t>
   </si>
   <si>
+    <t>RAKOTO Jean</t>
+  </si>
+  <si>
+    <t>033 12 345 67</t>
+  </si>
+  <si>
+    <t>Commerçant</t>
+  </si>
+  <si>
     <t>IF</t>
   </si>
   <si>
@@ -244,6 +268,15 @@
   </si>
   <si>
     <t>Morarano</t>
+  </si>
+  <si>
+    <t>RASOA Marie</t>
+  </si>
+  <si>
+    <t>034 98 765 43</t>
+  </si>
+  <si>
+    <t>Institutrice</t>
   </si>
   <si>
     <t>2024</t>
@@ -525,11 +558,14 @@
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -575,171 +611,206 @@
       <c r="N1" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="O1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>44</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J3" t="s">
-        <v>55</v>
-      </c>
-      <c r="K3" t="s">
-        <v>56</v>
+        <v>60</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>61</v>
       </c>
       <c r="L3" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="M3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N3" t="s">
-        <v>58</v>
+        <v>64</v>
+      </c>
+      <c r="O3" t="s">
+        <v>52</v>
+      </c>
+      <c r="P3" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E4" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="H4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s">
+        <v>74</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="M4" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" t="s">
+        <v>76</v>
+      </c>
+      <c r="O4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P4" t="s">
         <v>65</v>
       </c>
-      <c r="I4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J4" t="s">
-        <v>67</v>
-      </c>
-      <c r="K4" t="s">
-        <v>68</v>
-      </c>
-      <c r="L4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M4" t="s">
-        <v>57</v>
-      </c>
-      <c r="N4" t="s">
-        <v>47</v>
+      <c r="Q4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="I5" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="J5" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="L5" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="M5" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="N5" t="s">
-        <v>47</v>
+        <v>87</v>
+      </c>
+      <c r="O5" t="s">
+        <v>67</v>
+      </c>
+      <c r="P5" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -760,105 +831,105 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>